<commit_message>
feat(sdk): support multi-targeting net6.0;net7.0;net8.0 in ISC.Observability v1.5.0 & update tracking Excel
</commit_message>
<xml_diff>
--- a/docs/ISC_Form_Tracking_Observability_Services.xlsx
+++ b/docs/ISC_Form_Tracking_Observability_Services.xlsx
@@ -801,7 +801,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Số liệu tự động tổng hợp theo thời gian thực từ Sheet '02_TRACKING_SERVICES' (Dựa trên Quy định Observability v1.0 &amp; SDK v1.4.3)</t>
+          <t>Số liệu tự động tổng hợp theo thời gian thực từ Sheet '02_TRACKING_SERVICES' (Dựa trên Quy định Observability v1.0 &amp; SDK v1.5.0 Multi-Target .NET 6/7/8)</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
     <row r="26" ht="28" customHeight="1">
       <c r="B26" s="29" t="inlineStr">
         <is>
-          <t>IV. THỐNG KÊ THEO TECH STACK (ĐÁNH GIÁ ĐỘ PHỦ SDK .NET 8)</t>
+          <t>IV. THỐNG KÊ THEO TECH STACK (ĐÁNH GIÁ ĐỘ PHỦ SDK .NET 6 / 7 / 8)</t>
         </is>
       </c>
       <c r="C26" s="30" t="n"/>
@@ -1196,11 +1196,11 @@
     <row r="28" ht="24" customHeight="1">
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>.NET 8 (SDK hỗ trợ chính thức)</t>
+          <t>.NET 8 (SDK v1.5+ hỗ trợ chính thức)</t>
         </is>
       </c>
       <c r="C28" s="11">
-        <f>COUNTIF('02_TRACKING_SERVICES'!E6:E205, ".NET 8 (SDK hỗ trợ chính thức)")</f>
+        <f>COUNTIF('02_TRACKING_SERVICES'!E6:E205, ".NET 8 (SDK v1.5+ hỗ trợ chính thức)")</f>
         <v/>
       </c>
       <c r="D28" s="12">
@@ -1209,27 +1209,27 @@
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>Cài trực tiếp NuGet package ISC.Observability v1.4.3</t>
+          <t>Cài trực tiếp NuGet package ISC.Observability v1.5.0</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
-      <c r="B29" s="24" t="inlineStr">
-        <is>
-          <t>.NET 6 / .NET 7</t>
-        </is>
-      </c>
-      <c r="C29" s="25">
-        <f>COUNTIF('02_TRACKING_SERVICES'!E6:E205, ".NET 6 / .NET 7")</f>
-        <v/>
-      </c>
-      <c r="D29" s="26">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>.NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)</t>
+        </is>
+      </c>
+      <c r="C29" s="11">
+        <f>COUNTIF('02_TRACKING_SERVICES'!E6:E205, ".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)")</f>
+        <v/>
+      </c>
+      <c r="D29" s="12">
         <f>IF($C$6&gt;0, C29/$C$6, 0)</f>
         <v/>
       </c>
-      <c r="E29" s="24" t="inlineStr">
-        <is>
-          <t>Khuyến nghị nâng cấp .NET 8 hoặc dùng OTel Native</t>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Cài trực tiếp NuGet package ISC.Observability v1.5.0 (Multi-target)</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       <c r="F4" s="31" t="inlineStr">
         <is>
           <t>Khả năng hỗ trợ của SDK
-(Hiện chỉ hỗ trợ .NET 8)</t>
+(Hỗ trợ .NET 6 / 7 / 8)</t>
         </is>
       </c>
       <c r="G4" s="31" t="inlineStr">
@@ -1719,16 +1719,16 @@
       </c>
       <c r="E6" s="47" t="inlineStr">
         <is>
-          <t>.NET 8 (SDK hỗ trợ chính thức)</t>
+          <t>.NET 8 (SDK v1.5+ hỗ trợ chính thức)</t>
         </is>
       </c>
       <c r="F6" s="44">
-        <f>IF(E6="", "", IF(E6=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E6="", "", IF(OR(E6=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E6=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G6" s="47" t="inlineStr">
         <is>
-          <t>Đã cài SDK ISC.Observability (.NET 8)</t>
+          <t>Đã cài SDK ISC.Observability (.NET 6/7/8)</t>
         </is>
       </c>
       <c r="H6" s="47" t="inlineStr">
@@ -1826,16 +1826,16 @@
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>.NET 8 (SDK hỗ trợ chính thức)</t>
+          <t>.NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)</t>
         </is>
       </c>
       <c r="F7" s="44">
-        <f>IF(E7="", "", IF(E7=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E7="", "", IF(OR(E7=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E7=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>Đã cài SDK ISC.Observability (.NET 8)</t>
+          <t>Đã cài SDK ISC.Observability (.NET 6/7/8)</t>
         </is>
       </c>
       <c r="H7" s="25" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="V7" s="24" t="inlineStr">
         <is>
-          <t>Mẫu: Đang hoàn thiện custom metrics &amp; Dashboard Layer 3</t>
+          <t>Mẫu: Service .NET 6 cài trực tiếp SDK v1.5.0, đang hoàn thiện Dashboard Layer 3</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="F8" s="44">
-        <f>IF(E8="", "", IF(E8=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E8="", "", IF(OR(E8=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E8=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G8" s="47" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="Q8" s="47" t="inlineStr">
         <is>
-          <t>N/A (Ngoài .NET 8)</t>
+          <t>N/A (Ngoài .NET 6/7/8)</t>
         </is>
       </c>
       <c r="R8" s="44">
@@ -2040,11 +2040,11 @@
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
-          <t>.NET 6 / .NET 7</t>
+          <t>.NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)</t>
         </is>
       </c>
       <c r="F9" s="44">
-        <f>IF(E9="", "", IF(E9=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E9="", "", IF(OR(E9=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E9=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G9" s="25" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="V9" s="24" t="inlineStr">
         <is>
-          <t>Mẫu: Đang vi phạm đẩy log thẳng vào Kafka, chờ nâng cấp lên .NET 8</t>
+          <t>Mẫu: Đang vi phạm đẩy log thẳng vào Kafka, cần cài gói SDK v1.5.0 (.NET 6/7/8)</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="F10" s="44">
-        <f>IF(E10="", "", IF(E10=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E10="", "", IF(OR(E10=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E10=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G10" s="47" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="Q10" s="47" t="inlineStr">
         <is>
-          <t>N/A (Ngoài .NET 8)</t>
+          <t>N/A (Ngoài .NET 6/7/8)</t>
         </is>
       </c>
       <c r="R10" s="44">
@@ -2234,7 +2234,7 @@
       <c r="D11" s="25" t="n"/>
       <c r="E11" s="25" t="n"/>
       <c r="F11" s="44">
-        <f>IF(E11="", "", IF(E11=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E11="", "", IF(OR(E11=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E11=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G11" s="25" t="n"/>
@@ -2273,7 +2273,7 @@
       <c r="D12" s="47" t="n"/>
       <c r="E12" s="47" t="n"/>
       <c r="F12" s="44">
-        <f>IF(E12="", "", IF(E12=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E12="", "", IF(OR(E12=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E12=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G12" s="47" t="n"/>
@@ -2312,7 +2312,7 @@
       <c r="D13" s="25" t="n"/>
       <c r="E13" s="25" t="n"/>
       <c r="F13" s="44">
-        <f>IF(E13="", "", IF(E13=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E13="", "", IF(OR(E13=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E13=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G13" s="25" t="n"/>
@@ -2351,7 +2351,7 @@
       <c r="D14" s="47" t="n"/>
       <c r="E14" s="47" t="n"/>
       <c r="F14" s="44">
-        <f>IF(E14="", "", IF(E14=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E14="", "", IF(OR(E14=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E14=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G14" s="47" t="n"/>
@@ -2390,7 +2390,7 @@
       <c r="D15" s="25" t="n"/>
       <c r="E15" s="25" t="n"/>
       <c r="F15" s="44">
-        <f>IF(E15="", "", IF(E15=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E15="", "", IF(OR(E15=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E15=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G15" s="25" t="n"/>
@@ -2429,7 +2429,7 @@
       <c r="D16" s="47" t="n"/>
       <c r="E16" s="47" t="n"/>
       <c r="F16" s="44">
-        <f>IF(E16="", "", IF(E16=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E16="", "", IF(OR(E16=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E16=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G16" s="47" t="n"/>
@@ -2468,7 +2468,7 @@
       <c r="D17" s="25" t="n"/>
       <c r="E17" s="25" t="n"/>
       <c r="F17" s="44">
-        <f>IF(E17="", "", IF(E17=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E17="", "", IF(OR(E17=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E17=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G17" s="25" t="n"/>
@@ -2507,7 +2507,7 @@
       <c r="D18" s="47" t="n"/>
       <c r="E18" s="47" t="n"/>
       <c r="F18" s="44">
-        <f>IF(E18="", "", IF(E18=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E18="", "", IF(OR(E18=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E18=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G18" s="47" t="n"/>
@@ -2546,7 +2546,7 @@
       <c r="D19" s="25" t="n"/>
       <c r="E19" s="25" t="n"/>
       <c r="F19" s="44">
-        <f>IF(E19="", "", IF(E19=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E19="", "", IF(OR(E19=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E19=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G19" s="25" t="n"/>
@@ -2585,7 +2585,7 @@
       <c r="D20" s="47" t="n"/>
       <c r="E20" s="47" t="n"/>
       <c r="F20" s="44">
-        <f>IF(E20="", "", IF(E20=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E20="", "", IF(OR(E20=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E20=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G20" s="47" t="n"/>
@@ -2624,7 +2624,7 @@
       <c r="D21" s="25" t="n"/>
       <c r="E21" s="25" t="n"/>
       <c r="F21" s="44">
-        <f>IF(E21="", "", IF(E21=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E21="", "", IF(OR(E21=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E21=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G21" s="25" t="n"/>
@@ -2663,7 +2663,7 @@
       <c r="D22" s="47" t="n"/>
       <c r="E22" s="47" t="n"/>
       <c r="F22" s="44">
-        <f>IF(E22="", "", IF(E22=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E22="", "", IF(OR(E22=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E22=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G22" s="47" t="n"/>
@@ -2702,7 +2702,7 @@
       <c r="D23" s="25" t="n"/>
       <c r="E23" s="25" t="n"/>
       <c r="F23" s="44">
-        <f>IF(E23="", "", IF(E23=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E23="", "", IF(OR(E23=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E23=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G23" s="25" t="n"/>
@@ -2741,7 +2741,7 @@
       <c r="D24" s="47" t="n"/>
       <c r="E24" s="47" t="n"/>
       <c r="F24" s="44">
-        <f>IF(E24="", "", IF(E24=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E24="", "", IF(OR(E24=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E24=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G24" s="47" t="n"/>
@@ -2780,7 +2780,7 @@
       <c r="D25" s="25" t="n"/>
       <c r="E25" s="25" t="n"/>
       <c r="F25" s="44">
-        <f>IF(E25="", "", IF(E25=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E25="", "", IF(OR(E25=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E25=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G25" s="25" t="n"/>
@@ -2819,7 +2819,7 @@
       <c r="D26" s="47" t="n"/>
       <c r="E26" s="47" t="n"/>
       <c r="F26" s="44">
-        <f>IF(E26="", "", IF(E26=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E26="", "", IF(OR(E26=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E26=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G26" s="47" t="n"/>
@@ -2858,7 +2858,7 @@
       <c r="D27" s="25" t="n"/>
       <c r="E27" s="25" t="n"/>
       <c r="F27" s="44">
-        <f>IF(E27="", "", IF(E27=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E27="", "", IF(OR(E27=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E27=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G27" s="25" t="n"/>
@@ -2897,7 +2897,7 @@
       <c r="D28" s="47" t="n"/>
       <c r="E28" s="47" t="n"/>
       <c r="F28" s="44">
-        <f>IF(E28="", "", IF(E28=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E28="", "", IF(OR(E28=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E28=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G28" s="47" t="n"/>
@@ -2936,7 +2936,7 @@
       <c r="D29" s="25" t="n"/>
       <c r="E29" s="25" t="n"/>
       <c r="F29" s="44">
-        <f>IF(E29="", "", IF(E29=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E29="", "", IF(OR(E29=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E29=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G29" s="25" t="n"/>
@@ -2975,7 +2975,7 @@
       <c r="D30" s="47" t="n"/>
       <c r="E30" s="47" t="n"/>
       <c r="F30" s="44">
-        <f>IF(E30="", "", IF(E30=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E30="", "", IF(OR(E30=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E30=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G30" s="47" t="n"/>
@@ -3014,7 +3014,7 @@
       <c r="D31" s="25" t="n"/>
       <c r="E31" s="25" t="n"/>
       <c r="F31" s="44">
-        <f>IF(E31="", "", IF(E31=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E31="", "", IF(OR(E31=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E31=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G31" s="25" t="n"/>
@@ -3053,7 +3053,7 @@
       <c r="D32" s="47" t="n"/>
       <c r="E32" s="47" t="n"/>
       <c r="F32" s="44">
-        <f>IF(E32="", "", IF(E32=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E32="", "", IF(OR(E32=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E32=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G32" s="47" t="n"/>
@@ -3092,7 +3092,7 @@
       <c r="D33" s="25" t="n"/>
       <c r="E33" s="25" t="n"/>
       <c r="F33" s="44">
-        <f>IF(E33="", "", IF(E33=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E33="", "", IF(OR(E33=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E33=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G33" s="25" t="n"/>
@@ -3131,7 +3131,7 @@
       <c r="D34" s="47" t="n"/>
       <c r="E34" s="47" t="n"/>
       <c r="F34" s="44">
-        <f>IF(E34="", "", IF(E34=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E34="", "", IF(OR(E34=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E34=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G34" s="47" t="n"/>
@@ -3170,7 +3170,7 @@
       <c r="D35" s="25" t="n"/>
       <c r="E35" s="25" t="n"/>
       <c r="F35" s="44">
-        <f>IF(E35="", "", IF(E35=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E35="", "", IF(OR(E35=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E35=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G35" s="25" t="n"/>
@@ -3209,7 +3209,7 @@
       <c r="D36" s="47" t="n"/>
       <c r="E36" s="47" t="n"/>
       <c r="F36" s="44">
-        <f>IF(E36="", "", IF(E36=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E36="", "", IF(OR(E36=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E36=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G36" s="47" t="n"/>
@@ -3248,7 +3248,7 @@
       <c r="D37" s="25" t="n"/>
       <c r="E37" s="25" t="n"/>
       <c r="F37" s="44">
-        <f>IF(E37="", "", IF(E37=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E37="", "", IF(OR(E37=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E37=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G37" s="25" t="n"/>
@@ -3287,7 +3287,7 @@
       <c r="D38" s="47" t="n"/>
       <c r="E38" s="47" t="n"/>
       <c r="F38" s="44">
-        <f>IF(E38="", "", IF(E38=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E38="", "", IF(OR(E38=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E38=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G38" s="47" t="n"/>
@@ -3326,7 +3326,7 @@
       <c r="D39" s="25" t="n"/>
       <c r="E39" s="25" t="n"/>
       <c r="F39" s="44">
-        <f>IF(E39="", "", IF(E39=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E39="", "", IF(OR(E39=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E39=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G39" s="25" t="n"/>
@@ -3365,7 +3365,7 @@
       <c r="D40" s="47" t="n"/>
       <c r="E40" s="47" t="n"/>
       <c r="F40" s="44">
-        <f>IF(E40="", "", IF(E40=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E40="", "", IF(OR(E40=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E40=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G40" s="47" t="n"/>
@@ -3404,7 +3404,7 @@
       <c r="D41" s="25" t="n"/>
       <c r="E41" s="25" t="n"/>
       <c r="F41" s="44">
-        <f>IF(E41="", "", IF(E41=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E41="", "", IF(OR(E41=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E41=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G41" s="25" t="n"/>
@@ -3443,7 +3443,7 @@
       <c r="D42" s="47" t="n"/>
       <c r="E42" s="47" t="n"/>
       <c r="F42" s="44">
-        <f>IF(E42="", "", IF(E42=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E42="", "", IF(OR(E42=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E42=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G42" s="47" t="n"/>
@@ -3482,7 +3482,7 @@
       <c r="D43" s="25" t="n"/>
       <c r="E43" s="25" t="n"/>
       <c r="F43" s="44">
-        <f>IF(E43="", "", IF(E43=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E43="", "", IF(OR(E43=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E43=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G43" s="25" t="n"/>
@@ -3521,7 +3521,7 @@
       <c r="D44" s="47" t="n"/>
       <c r="E44" s="47" t="n"/>
       <c r="F44" s="44">
-        <f>IF(E44="", "", IF(E44=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E44="", "", IF(OR(E44=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E44=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G44" s="47" t="n"/>
@@ -3560,7 +3560,7 @@
       <c r="D45" s="25" t="n"/>
       <c r="E45" s="25" t="n"/>
       <c r="F45" s="44">
-        <f>IF(E45="", "", IF(E45=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E45="", "", IF(OR(E45=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E45=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G45" s="25" t="n"/>
@@ -3599,7 +3599,7 @@
       <c r="D46" s="47" t="n"/>
       <c r="E46" s="47" t="n"/>
       <c r="F46" s="44">
-        <f>IF(E46="", "", IF(E46=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E46="", "", IF(OR(E46=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E46=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G46" s="47" t="n"/>
@@ -3638,7 +3638,7 @@
       <c r="D47" s="25" t="n"/>
       <c r="E47" s="25" t="n"/>
       <c r="F47" s="44">
-        <f>IF(E47="", "", IF(E47=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E47="", "", IF(OR(E47=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E47=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G47" s="25" t="n"/>
@@ -3677,7 +3677,7 @@
       <c r="D48" s="47" t="n"/>
       <c r="E48" s="47" t="n"/>
       <c r="F48" s="44">
-        <f>IF(E48="", "", IF(E48=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E48="", "", IF(OR(E48=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E48=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G48" s="47" t="n"/>
@@ -3716,7 +3716,7 @@
       <c r="D49" s="25" t="n"/>
       <c r="E49" s="25" t="n"/>
       <c r="F49" s="44">
-        <f>IF(E49="", "", IF(E49=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E49="", "", IF(OR(E49=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E49=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G49" s="25" t="n"/>
@@ -3755,7 +3755,7 @@
       <c r="D50" s="47" t="n"/>
       <c r="E50" s="47" t="n"/>
       <c r="F50" s="44">
-        <f>IF(E50="", "", IF(E50=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E50="", "", IF(OR(E50=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E50=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G50" s="47" t="n"/>
@@ -3794,7 +3794,7 @@
       <c r="D51" s="25" t="n"/>
       <c r="E51" s="25" t="n"/>
       <c r="F51" s="44">
-        <f>IF(E51="", "", IF(E51=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E51="", "", IF(OR(E51=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E51=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G51" s="25" t="n"/>
@@ -3833,7 +3833,7 @@
       <c r="D52" s="47" t="n"/>
       <c r="E52" s="47" t="n"/>
       <c r="F52" s="44">
-        <f>IF(E52="", "", IF(E52=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E52="", "", IF(OR(E52=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E52=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G52" s="47" t="n"/>
@@ -3872,7 +3872,7 @@
       <c r="D53" s="25" t="n"/>
       <c r="E53" s="25" t="n"/>
       <c r="F53" s="44">
-        <f>IF(E53="", "", IF(E53=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E53="", "", IF(OR(E53=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E53=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G53" s="25" t="n"/>
@@ -3911,7 +3911,7 @@
       <c r="D54" s="47" t="n"/>
       <c r="E54" s="47" t="n"/>
       <c r="F54" s="44">
-        <f>IF(E54="", "", IF(E54=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E54="", "", IF(OR(E54=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E54=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G54" s="47" t="n"/>
@@ -3950,7 +3950,7 @@
       <c r="D55" s="25" t="n"/>
       <c r="E55" s="25" t="n"/>
       <c r="F55" s="44">
-        <f>IF(E55="", "", IF(E55=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E55="", "", IF(OR(E55=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E55=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G55" s="25" t="n"/>
@@ -3989,7 +3989,7 @@
       <c r="D56" s="47" t="n"/>
       <c r="E56" s="47" t="n"/>
       <c r="F56" s="44">
-        <f>IF(E56="", "", IF(E56=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E56="", "", IF(OR(E56=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E56=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G56" s="47" t="n"/>
@@ -4028,7 +4028,7 @@
       <c r="D57" s="25" t="n"/>
       <c r="E57" s="25" t="n"/>
       <c r="F57" s="44">
-        <f>IF(E57="", "", IF(E57=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E57="", "", IF(OR(E57=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E57=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G57" s="25" t="n"/>
@@ -4067,7 +4067,7 @@
       <c r="D58" s="47" t="n"/>
       <c r="E58" s="47" t="n"/>
       <c r="F58" s="44">
-        <f>IF(E58="", "", IF(E58=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E58="", "", IF(OR(E58=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E58=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G58" s="47" t="n"/>
@@ -4106,7 +4106,7 @@
       <c r="D59" s="25" t="n"/>
       <c r="E59" s="25" t="n"/>
       <c r="F59" s="44">
-        <f>IF(E59="", "", IF(E59=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E59="", "", IF(OR(E59=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E59=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G59" s="25" t="n"/>
@@ -4145,7 +4145,7 @@
       <c r="D60" s="47" t="n"/>
       <c r="E60" s="47" t="n"/>
       <c r="F60" s="44">
-        <f>IF(E60="", "", IF(E60=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E60="", "", IF(OR(E60=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E60=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G60" s="47" t="n"/>
@@ -4184,7 +4184,7 @@
       <c r="D61" s="25" t="n"/>
       <c r="E61" s="25" t="n"/>
       <c r="F61" s="44">
-        <f>IF(E61="", "", IF(E61=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E61="", "", IF(OR(E61=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E61=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G61" s="25" t="n"/>
@@ -4223,7 +4223,7 @@
       <c r="D62" s="47" t="n"/>
       <c r="E62" s="47" t="n"/>
       <c r="F62" s="44">
-        <f>IF(E62="", "", IF(E62=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E62="", "", IF(OR(E62=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E62=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G62" s="47" t="n"/>
@@ -4262,7 +4262,7 @@
       <c r="D63" s="25" t="n"/>
       <c r="E63" s="25" t="n"/>
       <c r="F63" s="44">
-        <f>IF(E63="", "", IF(E63=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E63="", "", IF(OR(E63=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E63=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G63" s="25" t="n"/>
@@ -4301,7 +4301,7 @@
       <c r="D64" s="47" t="n"/>
       <c r="E64" s="47" t="n"/>
       <c r="F64" s="44">
-        <f>IF(E64="", "", IF(E64=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E64="", "", IF(OR(E64=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E64=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G64" s="47" t="n"/>
@@ -4340,7 +4340,7 @@
       <c r="D65" s="25" t="n"/>
       <c r="E65" s="25" t="n"/>
       <c r="F65" s="44">
-        <f>IF(E65="", "", IF(E65=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E65="", "", IF(OR(E65=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E65=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G65" s="25" t="n"/>
@@ -4379,7 +4379,7 @@
       <c r="D66" s="47" t="n"/>
       <c r="E66" s="47" t="n"/>
       <c r="F66" s="44">
-        <f>IF(E66="", "", IF(E66=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E66="", "", IF(OR(E66=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E66=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G66" s="47" t="n"/>
@@ -4418,7 +4418,7 @@
       <c r="D67" s="25" t="n"/>
       <c r="E67" s="25" t="n"/>
       <c r="F67" s="44">
-        <f>IF(E67="", "", IF(E67=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E67="", "", IF(OR(E67=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E67=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G67" s="25" t="n"/>
@@ -4457,7 +4457,7 @@
       <c r="D68" s="47" t="n"/>
       <c r="E68" s="47" t="n"/>
       <c r="F68" s="44">
-        <f>IF(E68="", "", IF(E68=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E68="", "", IF(OR(E68=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E68=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G68" s="47" t="n"/>
@@ -4496,7 +4496,7 @@
       <c r="D69" s="25" t="n"/>
       <c r="E69" s="25" t="n"/>
       <c r="F69" s="44">
-        <f>IF(E69="", "", IF(E69=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E69="", "", IF(OR(E69=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E69=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G69" s="25" t="n"/>
@@ -4535,7 +4535,7 @@
       <c r="D70" s="47" t="n"/>
       <c r="E70" s="47" t="n"/>
       <c r="F70" s="44">
-        <f>IF(E70="", "", IF(E70=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E70="", "", IF(OR(E70=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E70=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G70" s="47" t="n"/>
@@ -4574,7 +4574,7 @@
       <c r="D71" s="25" t="n"/>
       <c r="E71" s="25" t="n"/>
       <c r="F71" s="44">
-        <f>IF(E71="", "", IF(E71=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E71="", "", IF(OR(E71=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E71=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G71" s="25" t="n"/>
@@ -4613,7 +4613,7 @@
       <c r="D72" s="47" t="n"/>
       <c r="E72" s="47" t="n"/>
       <c r="F72" s="44">
-        <f>IF(E72="", "", IF(E72=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E72="", "", IF(OR(E72=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E72=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G72" s="47" t="n"/>
@@ -4652,7 +4652,7 @@
       <c r="D73" s="25" t="n"/>
       <c r="E73" s="25" t="n"/>
       <c r="F73" s="44">
-        <f>IF(E73="", "", IF(E73=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E73="", "", IF(OR(E73=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E73=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G73" s="25" t="n"/>
@@ -4691,7 +4691,7 @@
       <c r="D74" s="47" t="n"/>
       <c r="E74" s="47" t="n"/>
       <c r="F74" s="44">
-        <f>IF(E74="", "", IF(E74=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E74="", "", IF(OR(E74=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E74=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G74" s="47" t="n"/>
@@ -4730,7 +4730,7 @@
       <c r="D75" s="25" t="n"/>
       <c r="E75" s="25" t="n"/>
       <c r="F75" s="44">
-        <f>IF(E75="", "", IF(E75=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E75="", "", IF(OR(E75=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E75=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G75" s="25" t="n"/>
@@ -4769,7 +4769,7 @@
       <c r="D76" s="47" t="n"/>
       <c r="E76" s="47" t="n"/>
       <c r="F76" s="44">
-        <f>IF(E76="", "", IF(E76=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E76="", "", IF(OR(E76=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E76=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G76" s="47" t="n"/>
@@ -4808,7 +4808,7 @@
       <c r="D77" s="25" t="n"/>
       <c r="E77" s="25" t="n"/>
       <c r="F77" s="44">
-        <f>IF(E77="", "", IF(E77=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E77="", "", IF(OR(E77=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E77=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G77" s="25" t="n"/>
@@ -4847,7 +4847,7 @@
       <c r="D78" s="47" t="n"/>
       <c r="E78" s="47" t="n"/>
       <c r="F78" s="44">
-        <f>IF(E78="", "", IF(E78=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E78="", "", IF(OR(E78=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E78=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G78" s="47" t="n"/>
@@ -4886,7 +4886,7 @@
       <c r="D79" s="25" t="n"/>
       <c r="E79" s="25" t="n"/>
       <c r="F79" s="44">
-        <f>IF(E79="", "", IF(E79=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E79="", "", IF(OR(E79=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E79=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G79" s="25" t="n"/>
@@ -4925,7 +4925,7 @@
       <c r="D80" s="47" t="n"/>
       <c r="E80" s="47" t="n"/>
       <c r="F80" s="44">
-        <f>IF(E80="", "", IF(E80=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E80="", "", IF(OR(E80=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E80=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G80" s="47" t="n"/>
@@ -4964,7 +4964,7 @@
       <c r="D81" s="25" t="n"/>
       <c r="E81" s="25" t="n"/>
       <c r="F81" s="44">
-        <f>IF(E81="", "", IF(E81=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E81="", "", IF(OR(E81=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E81=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G81" s="25" t="n"/>
@@ -5003,7 +5003,7 @@
       <c r="D82" s="47" t="n"/>
       <c r="E82" s="47" t="n"/>
       <c r="F82" s="44">
-        <f>IF(E82="", "", IF(E82=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E82="", "", IF(OR(E82=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E82=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G82" s="47" t="n"/>
@@ -5042,7 +5042,7 @@
       <c r="D83" s="25" t="n"/>
       <c r="E83" s="25" t="n"/>
       <c r="F83" s="44">
-        <f>IF(E83="", "", IF(E83=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E83="", "", IF(OR(E83=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E83=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G83" s="25" t="n"/>
@@ -5081,7 +5081,7 @@
       <c r="D84" s="47" t="n"/>
       <c r="E84" s="47" t="n"/>
       <c r="F84" s="44">
-        <f>IF(E84="", "", IF(E84=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E84="", "", IF(OR(E84=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E84=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G84" s="47" t="n"/>
@@ -5120,7 +5120,7 @@
       <c r="D85" s="25" t="n"/>
       <c r="E85" s="25" t="n"/>
       <c r="F85" s="44">
-        <f>IF(E85="", "", IF(E85=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E85="", "", IF(OR(E85=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E85=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G85" s="25" t="n"/>
@@ -5159,7 +5159,7 @@
       <c r="D86" s="47" t="n"/>
       <c r="E86" s="47" t="n"/>
       <c r="F86" s="44">
-        <f>IF(E86="", "", IF(E86=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E86="", "", IF(OR(E86=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E86=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G86" s="47" t="n"/>
@@ -5198,7 +5198,7 @@
       <c r="D87" s="25" t="n"/>
       <c r="E87" s="25" t="n"/>
       <c r="F87" s="44">
-        <f>IF(E87="", "", IF(E87=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E87="", "", IF(OR(E87=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E87=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G87" s="25" t="n"/>
@@ -5237,7 +5237,7 @@
       <c r="D88" s="47" t="n"/>
       <c r="E88" s="47" t="n"/>
       <c r="F88" s="44">
-        <f>IF(E88="", "", IF(E88=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E88="", "", IF(OR(E88=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E88=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G88" s="47" t="n"/>
@@ -5276,7 +5276,7 @@
       <c r="D89" s="25" t="n"/>
       <c r="E89" s="25" t="n"/>
       <c r="F89" s="44">
-        <f>IF(E89="", "", IF(E89=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E89="", "", IF(OR(E89=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E89=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G89" s="25" t="n"/>
@@ -5315,7 +5315,7 @@
       <c r="D90" s="47" t="n"/>
       <c r="E90" s="47" t="n"/>
       <c r="F90" s="44">
-        <f>IF(E90="", "", IF(E90=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E90="", "", IF(OR(E90=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E90=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G90" s="47" t="n"/>
@@ -5354,7 +5354,7 @@
       <c r="D91" s="25" t="n"/>
       <c r="E91" s="25" t="n"/>
       <c r="F91" s="44">
-        <f>IF(E91="", "", IF(E91=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E91="", "", IF(OR(E91=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E91=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G91" s="25" t="n"/>
@@ -5393,7 +5393,7 @@
       <c r="D92" s="47" t="n"/>
       <c r="E92" s="47" t="n"/>
       <c r="F92" s="44">
-        <f>IF(E92="", "", IF(E92=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E92="", "", IF(OR(E92=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E92=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G92" s="47" t="n"/>
@@ -5432,7 +5432,7 @@
       <c r="D93" s="25" t="n"/>
       <c r="E93" s="25" t="n"/>
       <c r="F93" s="44">
-        <f>IF(E93="", "", IF(E93=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E93="", "", IF(OR(E93=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E93=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G93" s="25" t="n"/>
@@ -5471,7 +5471,7 @@
       <c r="D94" s="47" t="n"/>
       <c r="E94" s="47" t="n"/>
       <c r="F94" s="44">
-        <f>IF(E94="", "", IF(E94=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E94="", "", IF(OR(E94=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E94=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G94" s="47" t="n"/>
@@ -5510,7 +5510,7 @@
       <c r="D95" s="25" t="n"/>
       <c r="E95" s="25" t="n"/>
       <c r="F95" s="44">
-        <f>IF(E95="", "", IF(E95=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E95="", "", IF(OR(E95=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E95=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G95" s="25" t="n"/>
@@ -5549,7 +5549,7 @@
       <c r="D96" s="47" t="n"/>
       <c r="E96" s="47" t="n"/>
       <c r="F96" s="44">
-        <f>IF(E96="", "", IF(E96=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E96="", "", IF(OR(E96=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E96=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G96" s="47" t="n"/>
@@ -5588,7 +5588,7 @@
       <c r="D97" s="25" t="n"/>
       <c r="E97" s="25" t="n"/>
       <c r="F97" s="44">
-        <f>IF(E97="", "", IF(E97=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E97="", "", IF(OR(E97=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E97=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G97" s="25" t="n"/>
@@ -5627,7 +5627,7 @@
       <c r="D98" s="47" t="n"/>
       <c r="E98" s="47" t="n"/>
       <c r="F98" s="44">
-        <f>IF(E98="", "", IF(E98=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E98="", "", IF(OR(E98=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E98=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G98" s="47" t="n"/>
@@ -5666,7 +5666,7 @@
       <c r="D99" s="25" t="n"/>
       <c r="E99" s="25" t="n"/>
       <c r="F99" s="44">
-        <f>IF(E99="", "", IF(E99=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E99="", "", IF(OR(E99=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E99=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G99" s="25" t="n"/>
@@ -5705,7 +5705,7 @@
       <c r="D100" s="47" t="n"/>
       <c r="E100" s="47" t="n"/>
       <c r="F100" s="44">
-        <f>IF(E100="", "", IF(E100=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E100="", "", IF(OR(E100=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E100=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G100" s="47" t="n"/>
@@ -5744,7 +5744,7 @@
       <c r="D101" s="25" t="n"/>
       <c r="E101" s="25" t="n"/>
       <c r="F101" s="44">
-        <f>IF(E101="", "", IF(E101=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E101="", "", IF(OR(E101=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E101=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G101" s="25" t="n"/>
@@ -5783,7 +5783,7 @@
       <c r="D102" s="47" t="n"/>
       <c r="E102" s="47" t="n"/>
       <c r="F102" s="44">
-        <f>IF(E102="", "", IF(E102=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E102="", "", IF(OR(E102=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E102=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G102" s="47" t="n"/>
@@ -5822,7 +5822,7 @@
       <c r="D103" s="25" t="n"/>
       <c r="E103" s="25" t="n"/>
       <c r="F103" s="44">
-        <f>IF(E103="", "", IF(E103=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E103="", "", IF(OR(E103=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E103=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G103" s="25" t="n"/>
@@ -5861,7 +5861,7 @@
       <c r="D104" s="47" t="n"/>
       <c r="E104" s="47" t="n"/>
       <c r="F104" s="44">
-        <f>IF(E104="", "", IF(E104=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E104="", "", IF(OR(E104=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E104=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G104" s="47" t="n"/>
@@ -5900,7 +5900,7 @@
       <c r="D105" s="25" t="n"/>
       <c r="E105" s="25" t="n"/>
       <c r="F105" s="44">
-        <f>IF(E105="", "", IF(E105=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E105="", "", IF(OR(E105=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E105=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G105" s="25" t="n"/>
@@ -5939,7 +5939,7 @@
       <c r="D106" s="47" t="n"/>
       <c r="E106" s="47" t="n"/>
       <c r="F106" s="44">
-        <f>IF(E106="", "", IF(E106=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E106="", "", IF(OR(E106=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E106=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G106" s="47" t="n"/>
@@ -5978,7 +5978,7 @@
       <c r="D107" s="25" t="n"/>
       <c r="E107" s="25" t="n"/>
       <c r="F107" s="44">
-        <f>IF(E107="", "", IF(E107=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E107="", "", IF(OR(E107=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E107=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G107" s="25" t="n"/>
@@ -6017,7 +6017,7 @@
       <c r="D108" s="47" t="n"/>
       <c r="E108" s="47" t="n"/>
       <c r="F108" s="44">
-        <f>IF(E108="", "", IF(E108=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E108="", "", IF(OR(E108=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E108=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G108" s="47" t="n"/>
@@ -6056,7 +6056,7 @@
       <c r="D109" s="25" t="n"/>
       <c r="E109" s="25" t="n"/>
       <c r="F109" s="44">
-        <f>IF(E109="", "", IF(E109=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E109="", "", IF(OR(E109=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E109=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G109" s="25" t="n"/>
@@ -6095,7 +6095,7 @@
       <c r="D110" s="47" t="n"/>
       <c r="E110" s="47" t="n"/>
       <c r="F110" s="44">
-        <f>IF(E110="", "", IF(E110=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E110="", "", IF(OR(E110=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E110=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G110" s="47" t="n"/>
@@ -6134,7 +6134,7 @@
       <c r="D111" s="25" t="n"/>
       <c r="E111" s="25" t="n"/>
       <c r="F111" s="44">
-        <f>IF(E111="", "", IF(E111=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E111="", "", IF(OR(E111=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E111=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G111" s="25" t="n"/>
@@ -6173,7 +6173,7 @@
       <c r="D112" s="47" t="n"/>
       <c r="E112" s="47" t="n"/>
       <c r="F112" s="44">
-        <f>IF(E112="", "", IF(E112=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E112="", "", IF(OR(E112=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E112=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G112" s="47" t="n"/>
@@ -6212,7 +6212,7 @@
       <c r="D113" s="25" t="n"/>
       <c r="E113" s="25" t="n"/>
       <c r="F113" s="44">
-        <f>IF(E113="", "", IF(E113=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E113="", "", IF(OR(E113=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E113=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G113" s="25" t="n"/>
@@ -6251,7 +6251,7 @@
       <c r="D114" s="47" t="n"/>
       <c r="E114" s="47" t="n"/>
       <c r="F114" s="44">
-        <f>IF(E114="", "", IF(E114=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E114="", "", IF(OR(E114=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E114=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G114" s="47" t="n"/>
@@ -6290,7 +6290,7 @@
       <c r="D115" s="25" t="n"/>
       <c r="E115" s="25" t="n"/>
       <c r="F115" s="44">
-        <f>IF(E115="", "", IF(E115=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E115="", "", IF(OR(E115=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E115=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G115" s="25" t="n"/>
@@ -6329,7 +6329,7 @@
       <c r="D116" s="47" t="n"/>
       <c r="E116" s="47" t="n"/>
       <c r="F116" s="44">
-        <f>IF(E116="", "", IF(E116=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E116="", "", IF(OR(E116=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E116=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G116" s="47" t="n"/>
@@ -6368,7 +6368,7 @@
       <c r="D117" s="25" t="n"/>
       <c r="E117" s="25" t="n"/>
       <c r="F117" s="44">
-        <f>IF(E117="", "", IF(E117=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E117="", "", IF(OR(E117=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E117=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G117" s="25" t="n"/>
@@ -6407,7 +6407,7 @@
       <c r="D118" s="47" t="n"/>
       <c r="E118" s="47" t="n"/>
       <c r="F118" s="44">
-        <f>IF(E118="", "", IF(E118=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E118="", "", IF(OR(E118=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E118=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G118" s="47" t="n"/>
@@ -6446,7 +6446,7 @@
       <c r="D119" s="25" t="n"/>
       <c r="E119" s="25" t="n"/>
       <c r="F119" s="44">
-        <f>IF(E119="", "", IF(E119=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E119="", "", IF(OR(E119=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E119=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G119" s="25" t="n"/>
@@ -6485,7 +6485,7 @@
       <c r="D120" s="47" t="n"/>
       <c r="E120" s="47" t="n"/>
       <c r="F120" s="44">
-        <f>IF(E120="", "", IF(E120=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E120="", "", IF(OR(E120=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E120=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G120" s="47" t="n"/>
@@ -6524,7 +6524,7 @@
       <c r="D121" s="25" t="n"/>
       <c r="E121" s="25" t="n"/>
       <c r="F121" s="44">
-        <f>IF(E121="", "", IF(E121=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E121="", "", IF(OR(E121=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E121=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G121" s="25" t="n"/>
@@ -6563,7 +6563,7 @@
       <c r="D122" s="47" t="n"/>
       <c r="E122" s="47" t="n"/>
       <c r="F122" s="44">
-        <f>IF(E122="", "", IF(E122=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E122="", "", IF(OR(E122=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E122=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G122" s="47" t="n"/>
@@ -6602,7 +6602,7 @@
       <c r="D123" s="25" t="n"/>
       <c r="E123" s="25" t="n"/>
       <c r="F123" s="44">
-        <f>IF(E123="", "", IF(E123=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E123="", "", IF(OR(E123=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E123=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G123" s="25" t="n"/>
@@ -6641,7 +6641,7 @@
       <c r="D124" s="47" t="n"/>
       <c r="E124" s="47" t="n"/>
       <c r="F124" s="44">
-        <f>IF(E124="", "", IF(E124=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E124="", "", IF(OR(E124=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E124=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G124" s="47" t="n"/>
@@ -6680,7 +6680,7 @@
       <c r="D125" s="25" t="n"/>
       <c r="E125" s="25" t="n"/>
       <c r="F125" s="44">
-        <f>IF(E125="", "", IF(E125=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E125="", "", IF(OR(E125=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E125=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G125" s="25" t="n"/>
@@ -6719,7 +6719,7 @@
       <c r="D126" s="47" t="n"/>
       <c r="E126" s="47" t="n"/>
       <c r="F126" s="44">
-        <f>IF(E126="", "", IF(E126=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E126="", "", IF(OR(E126=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E126=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G126" s="47" t="n"/>
@@ -6758,7 +6758,7 @@
       <c r="D127" s="25" t="n"/>
       <c r="E127" s="25" t="n"/>
       <c r="F127" s="44">
-        <f>IF(E127="", "", IF(E127=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E127="", "", IF(OR(E127=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E127=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G127" s="25" t="n"/>
@@ -6797,7 +6797,7 @@
       <c r="D128" s="47" t="n"/>
       <c r="E128" s="47" t="n"/>
       <c r="F128" s="44">
-        <f>IF(E128="", "", IF(E128=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E128="", "", IF(OR(E128=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E128=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G128" s="47" t="n"/>
@@ -6836,7 +6836,7 @@
       <c r="D129" s="25" t="n"/>
       <c r="E129" s="25" t="n"/>
       <c r="F129" s="44">
-        <f>IF(E129="", "", IF(E129=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E129="", "", IF(OR(E129=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E129=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G129" s="25" t="n"/>
@@ -6875,7 +6875,7 @@
       <c r="D130" s="47" t="n"/>
       <c r="E130" s="47" t="n"/>
       <c r="F130" s="44">
-        <f>IF(E130="", "", IF(E130=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E130="", "", IF(OR(E130=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E130=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G130" s="47" t="n"/>
@@ -6914,7 +6914,7 @@
       <c r="D131" s="25" t="n"/>
       <c r="E131" s="25" t="n"/>
       <c r="F131" s="44">
-        <f>IF(E131="", "", IF(E131=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E131="", "", IF(OR(E131=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E131=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G131" s="25" t="n"/>
@@ -6953,7 +6953,7 @@
       <c r="D132" s="47" t="n"/>
       <c r="E132" s="47" t="n"/>
       <c r="F132" s="44">
-        <f>IF(E132="", "", IF(E132=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E132="", "", IF(OR(E132=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E132=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G132" s="47" t="n"/>
@@ -6992,7 +6992,7 @@
       <c r="D133" s="25" t="n"/>
       <c r="E133" s="25" t="n"/>
       <c r="F133" s="44">
-        <f>IF(E133="", "", IF(E133=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E133="", "", IF(OR(E133=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E133=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G133" s="25" t="n"/>
@@ -7031,7 +7031,7 @@
       <c r="D134" s="47" t="n"/>
       <c r="E134" s="47" t="n"/>
       <c r="F134" s="44">
-        <f>IF(E134="", "", IF(E134=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E134="", "", IF(OR(E134=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E134=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G134" s="47" t="n"/>
@@ -7070,7 +7070,7 @@
       <c r="D135" s="25" t="n"/>
       <c r="E135" s="25" t="n"/>
       <c r="F135" s="44">
-        <f>IF(E135="", "", IF(E135=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E135="", "", IF(OR(E135=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E135=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G135" s="25" t="n"/>
@@ -7109,7 +7109,7 @@
       <c r="D136" s="47" t="n"/>
       <c r="E136" s="47" t="n"/>
       <c r="F136" s="44">
-        <f>IF(E136="", "", IF(E136=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E136="", "", IF(OR(E136=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E136=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G136" s="47" t="n"/>
@@ -7148,7 +7148,7 @@
       <c r="D137" s="25" t="n"/>
       <c r="E137" s="25" t="n"/>
       <c r="F137" s="44">
-        <f>IF(E137="", "", IF(E137=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E137="", "", IF(OR(E137=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E137=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G137" s="25" t="n"/>
@@ -7187,7 +7187,7 @@
       <c r="D138" s="47" t="n"/>
       <c r="E138" s="47" t="n"/>
       <c r="F138" s="44">
-        <f>IF(E138="", "", IF(E138=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E138="", "", IF(OR(E138=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E138=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G138" s="47" t="n"/>
@@ -7226,7 +7226,7 @@
       <c r="D139" s="25" t="n"/>
       <c r="E139" s="25" t="n"/>
       <c r="F139" s="44">
-        <f>IF(E139="", "", IF(E139=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E139="", "", IF(OR(E139=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E139=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G139" s="25" t="n"/>
@@ -7265,7 +7265,7 @@
       <c r="D140" s="47" t="n"/>
       <c r="E140" s="47" t="n"/>
       <c r="F140" s="44">
-        <f>IF(E140="", "", IF(E140=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E140="", "", IF(OR(E140=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E140=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G140" s="47" t="n"/>
@@ -7304,7 +7304,7 @@
       <c r="D141" s="25" t="n"/>
       <c r="E141" s="25" t="n"/>
       <c r="F141" s="44">
-        <f>IF(E141="", "", IF(E141=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E141="", "", IF(OR(E141=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E141=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G141" s="25" t="n"/>
@@ -7343,7 +7343,7 @@
       <c r="D142" s="47" t="n"/>
       <c r="E142" s="47" t="n"/>
       <c r="F142" s="44">
-        <f>IF(E142="", "", IF(E142=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E142="", "", IF(OR(E142=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E142=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G142" s="47" t="n"/>
@@ -7382,7 +7382,7 @@
       <c r="D143" s="25" t="n"/>
       <c r="E143" s="25" t="n"/>
       <c r="F143" s="44">
-        <f>IF(E143="", "", IF(E143=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E143="", "", IF(OR(E143=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E143=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G143" s="25" t="n"/>
@@ -7421,7 +7421,7 @@
       <c r="D144" s="47" t="n"/>
       <c r="E144" s="47" t="n"/>
       <c r="F144" s="44">
-        <f>IF(E144="", "", IF(E144=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E144="", "", IF(OR(E144=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E144=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G144" s="47" t="n"/>
@@ -7460,7 +7460,7 @@
       <c r="D145" s="25" t="n"/>
       <c r="E145" s="25" t="n"/>
       <c r="F145" s="44">
-        <f>IF(E145="", "", IF(E145=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E145="", "", IF(OR(E145=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E145=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G145" s="25" t="n"/>
@@ -7499,7 +7499,7 @@
       <c r="D146" s="47" t="n"/>
       <c r="E146" s="47" t="n"/>
       <c r="F146" s="44">
-        <f>IF(E146="", "", IF(E146=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E146="", "", IF(OR(E146=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E146=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G146" s="47" t="n"/>
@@ -7538,7 +7538,7 @@
       <c r="D147" s="25" t="n"/>
       <c r="E147" s="25" t="n"/>
       <c r="F147" s="44">
-        <f>IF(E147="", "", IF(E147=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E147="", "", IF(OR(E147=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E147=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G147" s="25" t="n"/>
@@ -7577,7 +7577,7 @@
       <c r="D148" s="47" t="n"/>
       <c r="E148" s="47" t="n"/>
       <c r="F148" s="44">
-        <f>IF(E148="", "", IF(E148=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E148="", "", IF(OR(E148=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E148=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G148" s="47" t="n"/>
@@ -7616,7 +7616,7 @@
       <c r="D149" s="25" t="n"/>
       <c r="E149" s="25" t="n"/>
       <c r="F149" s="44">
-        <f>IF(E149="", "", IF(E149=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E149="", "", IF(OR(E149=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E149=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G149" s="25" t="n"/>
@@ -7655,7 +7655,7 @@
       <c r="D150" s="47" t="n"/>
       <c r="E150" s="47" t="n"/>
       <c r="F150" s="44">
-        <f>IF(E150="", "", IF(E150=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E150="", "", IF(OR(E150=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E150=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G150" s="47" t="n"/>
@@ -7694,7 +7694,7 @@
       <c r="D151" s="25" t="n"/>
       <c r="E151" s="25" t="n"/>
       <c r="F151" s="44">
-        <f>IF(E151="", "", IF(E151=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E151="", "", IF(OR(E151=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E151=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G151" s="25" t="n"/>
@@ -7733,7 +7733,7 @@
       <c r="D152" s="47" t="n"/>
       <c r="E152" s="47" t="n"/>
       <c r="F152" s="44">
-        <f>IF(E152="", "", IF(E152=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E152="", "", IF(OR(E152=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E152=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G152" s="47" t="n"/>
@@ -7772,7 +7772,7 @@
       <c r="D153" s="25" t="n"/>
       <c r="E153" s="25" t="n"/>
       <c r="F153" s="44">
-        <f>IF(E153="", "", IF(E153=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E153="", "", IF(OR(E153=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E153=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G153" s="25" t="n"/>
@@ -7811,7 +7811,7 @@
       <c r="D154" s="47" t="n"/>
       <c r="E154" s="47" t="n"/>
       <c r="F154" s="44">
-        <f>IF(E154="", "", IF(E154=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E154="", "", IF(OR(E154=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E154=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G154" s="47" t="n"/>
@@ -7850,7 +7850,7 @@
       <c r="D155" s="25" t="n"/>
       <c r="E155" s="25" t="n"/>
       <c r="F155" s="44">
-        <f>IF(E155="", "", IF(E155=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E155="", "", IF(OR(E155=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E155=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G155" s="25" t="n"/>
@@ -7889,7 +7889,7 @@
       <c r="D156" s="47" t="n"/>
       <c r="E156" s="47" t="n"/>
       <c r="F156" s="44">
-        <f>IF(E156="", "", IF(E156=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E156="", "", IF(OR(E156=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E156=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G156" s="47" t="n"/>
@@ -7928,7 +7928,7 @@
       <c r="D157" s="25" t="n"/>
       <c r="E157" s="25" t="n"/>
       <c r="F157" s="44">
-        <f>IF(E157="", "", IF(E157=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E157="", "", IF(OR(E157=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E157=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G157" s="25" t="n"/>
@@ -7967,7 +7967,7 @@
       <c r="D158" s="47" t="n"/>
       <c r="E158" s="47" t="n"/>
       <c r="F158" s="44">
-        <f>IF(E158="", "", IF(E158=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E158="", "", IF(OR(E158=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E158=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G158" s="47" t="n"/>
@@ -8006,7 +8006,7 @@
       <c r="D159" s="25" t="n"/>
       <c r="E159" s="25" t="n"/>
       <c r="F159" s="44">
-        <f>IF(E159="", "", IF(E159=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E159="", "", IF(OR(E159=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E159=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G159" s="25" t="n"/>
@@ -8045,7 +8045,7 @@
       <c r="D160" s="47" t="n"/>
       <c r="E160" s="47" t="n"/>
       <c r="F160" s="44">
-        <f>IF(E160="", "", IF(E160=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E160="", "", IF(OR(E160=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E160=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G160" s="47" t="n"/>
@@ -8084,7 +8084,7 @@
       <c r="D161" s="25" t="n"/>
       <c r="E161" s="25" t="n"/>
       <c r="F161" s="44">
-        <f>IF(E161="", "", IF(E161=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E161="", "", IF(OR(E161=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E161=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G161" s="25" t="n"/>
@@ -8123,7 +8123,7 @@
       <c r="D162" s="47" t="n"/>
       <c r="E162" s="47" t="n"/>
       <c r="F162" s="44">
-        <f>IF(E162="", "", IF(E162=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E162="", "", IF(OR(E162=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E162=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G162" s="47" t="n"/>
@@ -8162,7 +8162,7 @@
       <c r="D163" s="25" t="n"/>
       <c r="E163" s="25" t="n"/>
       <c r="F163" s="44">
-        <f>IF(E163="", "", IF(E163=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E163="", "", IF(OR(E163=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E163=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G163" s="25" t="n"/>
@@ -8201,7 +8201,7 @@
       <c r="D164" s="47" t="n"/>
       <c r="E164" s="47" t="n"/>
       <c r="F164" s="44">
-        <f>IF(E164="", "", IF(E164=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E164="", "", IF(OR(E164=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E164=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G164" s="47" t="n"/>
@@ -8240,7 +8240,7 @@
       <c r="D165" s="25" t="n"/>
       <c r="E165" s="25" t="n"/>
       <c r="F165" s="44">
-        <f>IF(E165="", "", IF(E165=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E165="", "", IF(OR(E165=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E165=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G165" s="25" t="n"/>
@@ -8279,7 +8279,7 @@
       <c r="D166" s="47" t="n"/>
       <c r="E166" s="47" t="n"/>
       <c r="F166" s="44">
-        <f>IF(E166="", "", IF(E166=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E166="", "", IF(OR(E166=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E166=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G166" s="47" t="n"/>
@@ -8318,7 +8318,7 @@
       <c r="D167" s="25" t="n"/>
       <c r="E167" s="25" t="n"/>
       <c r="F167" s="44">
-        <f>IF(E167="", "", IF(E167=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E167="", "", IF(OR(E167=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E167=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G167" s="25" t="n"/>
@@ -8357,7 +8357,7 @@
       <c r="D168" s="47" t="n"/>
       <c r="E168" s="47" t="n"/>
       <c r="F168" s="44">
-        <f>IF(E168="", "", IF(E168=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E168="", "", IF(OR(E168=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E168=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G168" s="47" t="n"/>
@@ -8396,7 +8396,7 @@
       <c r="D169" s="25" t="n"/>
       <c r="E169" s="25" t="n"/>
       <c r="F169" s="44">
-        <f>IF(E169="", "", IF(E169=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E169="", "", IF(OR(E169=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E169=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G169" s="25" t="n"/>
@@ -8435,7 +8435,7 @@
       <c r="D170" s="47" t="n"/>
       <c r="E170" s="47" t="n"/>
       <c r="F170" s="44">
-        <f>IF(E170="", "", IF(E170=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E170="", "", IF(OR(E170=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E170=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G170" s="47" t="n"/>
@@ -8474,7 +8474,7 @@
       <c r="D171" s="25" t="n"/>
       <c r="E171" s="25" t="n"/>
       <c r="F171" s="44">
-        <f>IF(E171="", "", IF(E171=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E171="", "", IF(OR(E171=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E171=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G171" s="25" t="n"/>
@@ -8513,7 +8513,7 @@
       <c r="D172" s="47" t="n"/>
       <c r="E172" s="47" t="n"/>
       <c r="F172" s="44">
-        <f>IF(E172="", "", IF(E172=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E172="", "", IF(OR(E172=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E172=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G172" s="47" t="n"/>
@@ -8552,7 +8552,7 @@
       <c r="D173" s="25" t="n"/>
       <c r="E173" s="25" t="n"/>
       <c r="F173" s="44">
-        <f>IF(E173="", "", IF(E173=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E173="", "", IF(OR(E173=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E173=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G173" s="25" t="n"/>
@@ -8591,7 +8591,7 @@
       <c r="D174" s="47" t="n"/>
       <c r="E174" s="47" t="n"/>
       <c r="F174" s="44">
-        <f>IF(E174="", "", IF(E174=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E174="", "", IF(OR(E174=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E174=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G174" s="47" t="n"/>
@@ -8630,7 +8630,7 @@
       <c r="D175" s="25" t="n"/>
       <c r="E175" s="25" t="n"/>
       <c r="F175" s="44">
-        <f>IF(E175="", "", IF(E175=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E175="", "", IF(OR(E175=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E175=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G175" s="25" t="n"/>
@@ -8669,7 +8669,7 @@
       <c r="D176" s="47" t="n"/>
       <c r="E176" s="47" t="n"/>
       <c r="F176" s="44">
-        <f>IF(E176="", "", IF(E176=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E176="", "", IF(OR(E176=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E176=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G176" s="47" t="n"/>
@@ -8708,7 +8708,7 @@
       <c r="D177" s="25" t="n"/>
       <c r="E177" s="25" t="n"/>
       <c r="F177" s="44">
-        <f>IF(E177="", "", IF(E177=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E177="", "", IF(OR(E177=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E177=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G177" s="25" t="n"/>
@@ -8747,7 +8747,7 @@
       <c r="D178" s="47" t="n"/>
       <c r="E178" s="47" t="n"/>
       <c r="F178" s="44">
-        <f>IF(E178="", "", IF(E178=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E178="", "", IF(OR(E178=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E178=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G178" s="47" t="n"/>
@@ -8786,7 +8786,7 @@
       <c r="D179" s="25" t="n"/>
       <c r="E179" s="25" t="n"/>
       <c r="F179" s="44">
-        <f>IF(E179="", "", IF(E179=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E179="", "", IF(OR(E179=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E179=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G179" s="25" t="n"/>
@@ -8825,7 +8825,7 @@
       <c r="D180" s="47" t="n"/>
       <c r="E180" s="47" t="n"/>
       <c r="F180" s="44">
-        <f>IF(E180="", "", IF(E180=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E180="", "", IF(OR(E180=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E180=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G180" s="47" t="n"/>
@@ -8864,7 +8864,7 @@
       <c r="D181" s="25" t="n"/>
       <c r="E181" s="25" t="n"/>
       <c r="F181" s="44">
-        <f>IF(E181="", "", IF(E181=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E181="", "", IF(OR(E181=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E181=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G181" s="25" t="n"/>
@@ -8903,7 +8903,7 @@
       <c r="D182" s="47" t="n"/>
       <c r="E182" s="47" t="n"/>
       <c r="F182" s="44">
-        <f>IF(E182="", "", IF(E182=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E182="", "", IF(OR(E182=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E182=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G182" s="47" t="n"/>
@@ -8942,7 +8942,7 @@
       <c r="D183" s="25" t="n"/>
       <c r="E183" s="25" t="n"/>
       <c r="F183" s="44">
-        <f>IF(E183="", "", IF(E183=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E183="", "", IF(OR(E183=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E183=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G183" s="25" t="n"/>
@@ -8981,7 +8981,7 @@
       <c r="D184" s="47" t="n"/>
       <c r="E184" s="47" t="n"/>
       <c r="F184" s="44">
-        <f>IF(E184="", "", IF(E184=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E184="", "", IF(OR(E184=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E184=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G184" s="47" t="n"/>
@@ -9020,7 +9020,7 @@
       <c r="D185" s="25" t="n"/>
       <c r="E185" s="25" t="n"/>
       <c r="F185" s="44">
-        <f>IF(E185="", "", IF(E185=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E185="", "", IF(OR(E185=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E185=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G185" s="25" t="n"/>
@@ -9059,7 +9059,7 @@
       <c r="D186" s="47" t="n"/>
       <c r="E186" s="47" t="n"/>
       <c r="F186" s="44">
-        <f>IF(E186="", "", IF(E186=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E186="", "", IF(OR(E186=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E186=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G186" s="47" t="n"/>
@@ -9098,7 +9098,7 @@
       <c r="D187" s="25" t="n"/>
       <c r="E187" s="25" t="n"/>
       <c r="F187" s="44">
-        <f>IF(E187="", "", IF(E187=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E187="", "", IF(OR(E187=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E187=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G187" s="25" t="n"/>
@@ -9137,7 +9137,7 @@
       <c r="D188" s="47" t="n"/>
       <c r="E188" s="47" t="n"/>
       <c r="F188" s="44">
-        <f>IF(E188="", "", IF(E188=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E188="", "", IF(OR(E188=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E188=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G188" s="47" t="n"/>
@@ -9176,7 +9176,7 @@
       <c r="D189" s="25" t="n"/>
       <c r="E189" s="25" t="n"/>
       <c r="F189" s="44">
-        <f>IF(E189="", "", IF(E189=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E189="", "", IF(OR(E189=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E189=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G189" s="25" t="n"/>
@@ -9215,7 +9215,7 @@
       <c r="D190" s="47" t="n"/>
       <c r="E190" s="47" t="n"/>
       <c r="F190" s="44">
-        <f>IF(E190="", "", IF(E190=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E190="", "", IF(OR(E190=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E190=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G190" s="47" t="n"/>
@@ -9254,7 +9254,7 @@
       <c r="D191" s="25" t="n"/>
       <c r="E191" s="25" t="n"/>
       <c r="F191" s="44">
-        <f>IF(E191="", "", IF(E191=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E191="", "", IF(OR(E191=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E191=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G191" s="25" t="n"/>
@@ -9293,7 +9293,7 @@
       <c r="D192" s="47" t="n"/>
       <c r="E192" s="47" t="n"/>
       <c r="F192" s="44">
-        <f>IF(E192="", "", IF(E192=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E192="", "", IF(OR(E192=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E192=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G192" s="47" t="n"/>
@@ -9332,7 +9332,7 @@
       <c r="D193" s="25" t="n"/>
       <c r="E193" s="25" t="n"/>
       <c r="F193" s="44">
-        <f>IF(E193="", "", IF(E193=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E193="", "", IF(OR(E193=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E193=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G193" s="25" t="n"/>
@@ -9371,7 +9371,7 @@
       <c r="D194" s="47" t="n"/>
       <c r="E194" s="47" t="n"/>
       <c r="F194" s="44">
-        <f>IF(E194="", "", IF(E194=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E194="", "", IF(OR(E194=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E194=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G194" s="47" t="n"/>
@@ -9410,7 +9410,7 @@
       <c r="D195" s="25" t="n"/>
       <c r="E195" s="25" t="n"/>
       <c r="F195" s="44">
-        <f>IF(E195="", "", IF(E195=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E195="", "", IF(OR(E195=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E195=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G195" s="25" t="n"/>
@@ -9449,7 +9449,7 @@
       <c r="D196" s="47" t="n"/>
       <c r="E196" s="47" t="n"/>
       <c r="F196" s="44">
-        <f>IF(E196="", "", IF(E196=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E196="", "", IF(OR(E196=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E196=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G196" s="47" t="n"/>
@@ -9488,7 +9488,7 @@
       <c r="D197" s="25" t="n"/>
       <c r="E197" s="25" t="n"/>
       <c r="F197" s="44">
-        <f>IF(E197="", "", IF(E197=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E197="", "", IF(OR(E197=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E197=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G197" s="25" t="n"/>
@@ -9527,7 +9527,7 @@
       <c r="D198" s="47" t="n"/>
       <c r="E198" s="47" t="n"/>
       <c r="F198" s="44">
-        <f>IF(E198="", "", IF(E198=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E198="", "", IF(OR(E198=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E198=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G198" s="47" t="n"/>
@@ -9566,7 +9566,7 @@
       <c r="D199" s="25" t="n"/>
       <c r="E199" s="25" t="n"/>
       <c r="F199" s="44">
-        <f>IF(E199="", "", IF(E199=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E199="", "", IF(OR(E199=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E199=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G199" s="25" t="n"/>
@@ -9605,7 +9605,7 @@
       <c r="D200" s="47" t="n"/>
       <c r="E200" s="47" t="n"/>
       <c r="F200" s="44">
-        <f>IF(E200="", "", IF(E200=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E200="", "", IF(OR(E200=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E200=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G200" s="47" t="n"/>
@@ -9644,7 +9644,7 @@
       <c r="D201" s="25" t="n"/>
       <c r="E201" s="25" t="n"/>
       <c r="F201" s="44">
-        <f>IF(E201="", "", IF(E201=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E201="", "", IF(OR(E201=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E201=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G201" s="25" t="n"/>
@@ -9683,7 +9683,7 @@
       <c r="D202" s="47" t="n"/>
       <c r="E202" s="47" t="n"/>
       <c r="F202" s="44">
-        <f>IF(E202="", "", IF(E202=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E202="", "", IF(OR(E202=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E202=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G202" s="47" t="n"/>
@@ -9722,7 +9722,7 @@
       <c r="D203" s="25" t="n"/>
       <c r="E203" s="25" t="n"/>
       <c r="F203" s="44">
-        <f>IF(E203="", "", IF(E203=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E203="", "", IF(OR(E203=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E203=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G203" s="25" t="n"/>
@@ -9761,7 +9761,7 @@
       <c r="D204" s="47" t="n"/>
       <c r="E204" s="47" t="n"/>
       <c r="F204" s="44">
-        <f>IF(E204="", "", IF(E204=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E204="", "", IF(OR(E204=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E204=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G204" s="47" t="n"/>
@@ -9800,7 +9800,7 @@
       <c r="D205" s="25" t="n"/>
       <c r="E205" s="25" t="n"/>
       <c r="F205" s="44">
-        <f>IF(E205="", "", IF(E205=".NET 8 (SDK hỗ trợ chính thức)", "Hỗ trợ chuẩn SDK (.NET 8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
+        <f>IF(E205="", "", IF(OR(E205=".NET 8 (SDK v1.5+ hỗ trợ chính thức)", E205=".NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)"), "Hỗ trợ chuẩn SDK (.NET 6/7/8)", "Ngoài phạm vi SDK (Dùng OTel Native)"))</f>
         <v/>
       </c>
       <c r="G205" s="25" t="n"/>
@@ -9863,10 +9863,10 @@
       <formula>"ĐẠT CHUẨN QG2 (PASS)"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="0" stopIfTrue="1">
-      <formula>"Hỗ trợ chuẩn SDK (.NET 8)"</formula>
+      <formula>"Hỗ trợ chuẩn SDK (.NET 6/7/8)"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="9" operator="equal" dxfId="0" stopIfTrue="1">
-      <formula>"Đã cài SDK ISC.Observability (.NET 8)"</formula>
+      <formula>"Đã cài SDK ISC.Observability (.NET 6/7/8)"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="1" stopIfTrue="1">
       <formula>"Đẩy thẳng Kafka / ES (Vi phạm BLOCKER)"</formula>
@@ -9921,7 +9921,7 @@
     <dataValidation sqref="D6:D205" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Chọn Môi trường" prompt="Vui lòng chọn môi trường từ danh sách" type="list">
       <formula1>='03_DANH_MUC_CHUAN'!$B$4:$B$7</formula1>
     </dataValidation>
-    <dataValidation sqref="E6:E205" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Chọn Tech Stack" prompt="Hiện tại SDK chỉ hỗ trợ chính thức .NET 8" type="list">
+    <dataValidation sqref="E6:E205" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Chọn Tech Stack" prompt="SDK v1.5.0+ hỗ trợ chính thức .NET 6, .NET 7 và .NET 8" type="list">
       <formula1>='03_DANH_MUC_CHUAN'!$A$4:$A$11</formula1>
     </dataValidation>
     <dataValidation sqref="G6:G205" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Chọn Phương thức tích hợp" prompt="Chọn phương thức tích hợp" type="list">
@@ -10021,7 +10021,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="49" t="inlineStr">
         <is>
-          <t>.NET 8 (SDK hỗ trợ chính thức)</t>
+          <t>.NET 8 (SDK v1.5+ hỗ trợ chính thức)</t>
         </is>
       </c>
       <c r="B4" s="49" t="inlineStr">
@@ -10031,7 +10031,7 @@
       </c>
       <c r="C4" s="49" t="inlineStr">
         <is>
-          <t>Đã cài SDK ISC.Observability (.NET 8)</t>
+          <t>Đã cài SDK ISC.Observability (.NET 6/7/8)</t>
         </is>
       </c>
       <c r="D4" s="49" t="inlineStr">
@@ -10058,7 +10058,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="49" t="inlineStr">
         <is>
-          <t>.NET 6 / .NET 7</t>
+          <t>.NET 6 / .NET 7 (SDK v1.5+ hỗ trợ chính thức)</t>
         </is>
       </c>
       <c r="B5" s="49" t="inlineStr">
@@ -10125,7 +10125,7 @@
       </c>
       <c r="G6" s="49" t="inlineStr">
         <is>
-          <t>N/A (Ngoài .NET 8)</t>
+          <t>N/A (Ngoài .NET 6/7/8)</t>
         </is>
       </c>
     </row>
@@ -10206,7 +10206,7 @@
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Cơ chế hỗ trợ trong SDK (.NET 8)</t>
+          <t>Cơ chế hỗ trợ trong SDK (.NET 6 / 7 / 8)</t>
         </is>
       </c>
       <c r="F15" s="5" t="n"/>

</xml_diff>